<commit_message>
Implement prompt instruction judge metrics
</commit_message>
<xml_diff>
--- a/docs/COMBINED_JUDGE_METRICS.xlsx
+++ b/docs/COMBINED_JUDGE_METRICS.xlsx
@@ -101,7 +101,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -123,11 +123,55 @@
         <color rgb="00D9E2F3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -160,6 +204,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1250,58 +1297,58 @@
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>instruction_adherence_score</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>LLM judge + rule</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>0.0 ~ 1.0</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Agent가 주어진 instruction을 따른 정도.</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>계획 지표: detector 구현 및 trace event 수집 필요</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>score &lt; 1.0 or violations present</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="n">
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2322,120 +2369,120 @@
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>output_format_compliance</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>deterministic parser</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>요구된 output format을 지켰는지.</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>계획 지표: detector 구현 및 trace event 수집 필요</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>required output format is not compliant</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>prompt_template_version_present</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>trace 검사</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>존재 여부</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>trace에 prompt template 이름/version이 기록되어 있는지.</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>계획 지표: detector 구현 및 trace event 수집 필요</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>prompt template name/version missing</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2755,7 +2802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2836,442 +2883,607 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>output_contract_compliance</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>final output이 markdown contract를 만족하는지.</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>deterministic parser</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>critical/high</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="12" t="inlineStr">
         <is>
           <t>output_contract()</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="12" t="inlineStr">
         <is>
           <t>final_output</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>final_output.content</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="12" t="inlineStr">
         <is>
           <t>final_output 누락/공백 또는 필수 Markdown 섹션 누락</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>target_endpoint_consistency</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>사용자 요청 target endpoint와 tool/metric path가 일치하는지.</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>rule (context)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>wrong_endpoint()</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="12" t="inlineStr">
         <is>
           <t>run_start/chat_turn_start, tool_start, tool_end</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>user_input, filter_log_records.path_pattern, compute_log_metrics.top_paths[].path</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="12" t="inlineStr">
         <is>
           <t>사용자 요청 target path와 tool argument/metric path 불일치</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>metric_result_consistency</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>metric claim이 검증 가능한 tool output에서 왔는지.</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>rule (tool output)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>metric_consistency()</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>react_step, tool_end, node_start, node_end</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>react_step.action, tool_end.tool, state.metrics.faultInjected</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>compute step은 있으나 compute_log_metrics tool_end가 없거나, faultInjected metrics 사용</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>validation_path_coverage</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>validate_findings node와 validation_result가 실행되었는지.</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>rule (expected path)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>validation_path()</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>node_start, validation_result, edge_selected</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>node_start.node, validation_result count, edge_selected.reason</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>validate_findings node/result 누락 또는 validation skip edge 감지</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>parse_error_handling_score</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>높은 parse error ratio를 차단/반영했는지.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>0.0 ~ 1.0</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>parse_error_handling()</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>tool_end(parse_access_log), final_output, validation_result</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>parse_error_count, total_lines, final_output.content, validation_result.issues</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="12" t="inlineStr">
         <is>
           <t>parse_error_count / total_lines &gt; 0.5</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>rag_context_presence_and_usage</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>RAG retrieval과 final report 반영 여부.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>rag_mcp_presence()</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>tool_end, final_output</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>tool_end.tool, final_output.content</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="12" t="inlineStr">
         <is>
           <t>retrieve_runbook 누락 또는 final report의 ## RAG Context 섹션 누락</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>instruction_adherence_score</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Agent가 주어진 instruction을 따른 정도.</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>LLM judge + rule</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>0.0 ~ 1.0</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>instruction_adherence()</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>prompt_instruction_metrics</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>instruction_adherence.score, instruction_adherence.violations</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>score &lt; 1.0 or violations present</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>mcp_context_presence_and_usage</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>MCP service context 수집과 final report 반영 여부.</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>rag_mcp_presence()</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
         <is>
           <t>mcp_end, final_output</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>mcp_end.method, final_output.content</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K10" s="12" t="inlineStr">
         <is>
           <t>mcp_end tools/call 누락 또는 final report의 ## MCP Context 섹션 누락</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>chat_context_grounding</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>후속 대화가 직전 analysis/focus/evidence에 grounded 되었는지.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>pass/fail</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>medium/low</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>chat_context()</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>chat_*, chat_analysis_invoked, chat_context_built, chat_response_generated</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>chat_context_built.has_last_analysis</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>후속 대화가 last analysis/context evidence에 grounded 되지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>output_format_compliance</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>요구된 output format을 지켰는지.</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>deterministic parser</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>pass/fail</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>output_format_compliance()</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>prompt_instruction_metrics, final_output fallback</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>output_format.compliant, output_format.missing_sections</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>required output format is not compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>prompt_template_version_present</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>trace에 prompt template 이름/version이 기록되어 있는지.</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>trace 검사</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>존재 여부</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>prompt_template_version()</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>instruction_snapshot, prompt_instruction_metrics</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>prompt_template.name, prompt_template.version, prompt_template.present</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>prompt template name/version missing</t>
         </is>
       </c>
     </row>
@@ -4033,47 +4245,47 @@
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>instruction_adherence_score</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Agent가 주어진 instruction을 따른 정도.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>LLM judge + rule</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>0.0 ~ 1.0</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -4169,6 +4381,10 @@
 validation path 누락/skip</t>
         </is>
       </c>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="14" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -4187,6 +4403,10 @@
 target endpoint 불일치 / metric result 불일치</t>
         </is>
       </c>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="14" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -4204,6 +4424,10 @@
 근거 부족한 follow-up 응답</t>
         </is>
       </c>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="14" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -4219,6 +4443,10 @@
 낮은 신뢰도의 context grounding warning</t>
         </is>
       </c>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="14" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">

</xml_diff>